<commit_message>
v2.9: fix - 2026/06/18
</commit_message>
<xml_diff>
--- a/resources/M673/M673_codebaseline.xlsx
+++ b/resources/M673/M673_codebaseline.xlsx
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.00316</v>
+        <v>0.00317</v>
       </c>
     </row>
     <row r="3">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.00143</v>
+        <v>0.00144</v>
       </c>
     </row>
     <row r="6">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.01206</v>
+        <v>0.008460000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00362</v>
+        <v>0.00363</v>
       </c>
     </row>
     <row r="19">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.00148</v>
+        <v>0.00149</v>
       </c>
     </row>
     <row r="26">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.00038</v>
+        <v>0.00076</v>
       </c>
     </row>
     <row r="29">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="30">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.00229</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="34">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.00054</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="35">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.00377</v>
+        <v>0.00302</v>
       </c>
     </row>
     <row r="36">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.00447</v>
+        <v>0.00449</v>
       </c>
     </row>
     <row r="41">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.00327</v>
+        <v>0.00328</v>
       </c>
     </row>
     <row r="49">
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.00405</v>
+        <v>0.00541</v>
       </c>
     </row>
   </sheetData>
@@ -967,7 +967,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-18T09:30:31.520752</t>
+          <t>2026-06-18T09:51:49.490807</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>G向ELA Mura=0;S向ELA Mura=0;大面积亮点=0.5;大面积暗点=0.5;暗点=1.5;群暗点=1.5</t>
+          <t>G向ELA Mura=0;S向ELA Mura=0;S向亮线=0.7;彩斑Mura=0.8;暗点=1.5;群暗点=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.9: fix - 20260630
</commit_message>
<xml_diff>
--- a/resources/M673/M673_codebaseline.xlsx
+++ b/resources/M673/M673_codebaseline.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.00317</v>
+        <v>0.00456</v>
       </c>
     </row>
     <row r="3">
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5e-05</v>
+        <v>6e-05</v>
       </c>
     </row>
     <row r="4">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.00085</v>
+        <v>0.00092</v>
       </c>
     </row>
     <row r="5">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.00144</v>
+        <v>0.00143</v>
       </c>
     </row>
     <row r="6">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1e-05</v>
+        <v>2e-05</v>
       </c>
     </row>
     <row r="7">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00015</v>
+        <v>0.00019</v>
       </c>
     </row>
     <row r="8">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.999999999999999e-05</v>
+        <v>0.00011</v>
       </c>
     </row>
     <row r="10">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2e-05</v>
+        <v>3e-05</v>
       </c>
     </row>
     <row r="11">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00024</v>
+        <v>0.00027</v>
       </c>
     </row>
     <row r="12">
@@ -554,187 +554,187 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>L3亮点</t>
+          <t>IC侧 Mura</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.00012</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PCD裂纹亮线</t>
+          <t>IC侧长条形Mura</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RGB亮点</t>
+          <t>L3亮点</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6e-05</v>
+        <v>0.00041</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RGB黑斑</t>
+          <t>PCD裂纹亮线</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2e-05</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S向亮线</t>
+          <t>RGB亮点</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.008460000000000001</v>
+        <v>0.00013</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S向单暗线</t>
+          <t>RGB黑斑</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00363</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S向带状Mura</t>
+          <t>S向亮线</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.00017</v>
+        <v>0.00728</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S向彩色带状Mura</t>
+          <t>S向单暗线</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1e-05</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S向微亮线</t>
+          <t>S向带状Mura</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3e-05</v>
+        <v>0.00016</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S向棱形彩色带状Mura</t>
+          <t>S向彩色带状Mura</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.00043</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S向群亮线</t>
+          <t>S向微亮线</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0001</v>
+        <v>3e-05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S向边缘Mura</t>
+          <t>S向棱形彩色带状Mura</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.00035</v>
+        <v>0.00044</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>单亮点</t>
+          <t>S向群亮线</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.00149</v>
+        <v>9.000000000000001e-05</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>可修复暗点</t>
+          <t>S向群暗线</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3e-05</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>大圆环Mura</t>
+          <t>S向边缘Mura</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1e-05</v>
+        <v>0.00037</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>大面积亮点</t>
+          <t>单亮点</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.00076</v>
+        <v>0.00163</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>大面积暗点</t>
+          <t>可修复亮点</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>大面积片状彩斑Mura</t>
+          <t>可修复暗点</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>3e-05</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>孔区跑道Mura</t>
+          <t>大圆环Mura</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -744,57 +744,57 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>左斜黑色带状Mura</t>
+          <t>大面积亮点</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1e-05</v>
+        <v>0.00092</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>常亮白斑</t>
+          <t>大面积暗点</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.0023</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>常暗黑斑Mura</t>
+          <t>大面积片状彩斑Mura</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.00055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>彩斑Mura</t>
+          <t>孔区环状Mura</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.00302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>微亮点</t>
+          <t>孔区跑道Mura</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.00018</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>微暗点</t>
+          <t>左斜黑色带状Mura</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -804,67 +804,67 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>摩尔纹</t>
+          <t>常亮白斑</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>0.00444</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>斑中带点</t>
+          <t>常暗黑斑Mura</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1e-05</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>暗点</t>
+          <t>彩斑Mura</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.00449</v>
+        <v>0.00537</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>流星状划线</t>
+          <t>微亮点</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2e-05</v>
+        <v>0.00017</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>灰阶块状白斑Mura</t>
+          <t>微暗点</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>1e-05</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>灰阶小白斑Mura</t>
+          <t>摩尔纹</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>灰阶暗点</t>
+          <t>斑中带点</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -874,51 +874,111 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>灰阶点状白斑Mura</t>
+          <t>暗点</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0</v>
+        <v>0.00779</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>环状Mura</t>
+          <t>流星状划线</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>3e-05</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>白画面黑斑Mura</t>
+          <t>灰阶块状白斑Mura</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.00119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>群亮点</t>
+          <t>灰阶小白斑Mura</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.00328</v>
+        <v>8.000000000000001e-05</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>灰阶暗点</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2e-05</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>灰阶点状白斑Mura</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1e-05</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>环状Mura</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2e-05</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>白画面黑斑Mura</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.00187</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>群亮点</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.00647</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>群暗点</t>
         </is>
       </c>
-      <c r="B49" t="n">
-        <v>0.00541</v>
+      <c r="B54" t="n">
+        <v>0.00458</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>雪花状Mura</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -967,7 +1027,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-18T09:51:49.490807</t>
+          <t>2026-06-30T11:38:51.331457</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1075,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1087,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>54</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1099,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>G向ELA Mura=0;S向ELA Mura=0;S向亮线=0.7;彩斑Mura=0.8;暗点=1.5;群暗点=2</t>
+          <t>G向ELA Mura=0;S向ELA Mura=0;S向亮线=0.7;暗点=1.8;群亮点=1.2;群暗点=1.2</t>
         </is>
       </c>
     </row>

</xml_diff>